<commit_message>
Following register by register confirmation for PQ1 registers.  Updates to documentation and entity descriptions
</commit_message>
<xml_diff>
--- a/docs/FoxESS_PQ1_Register_Mapping_and_Test_Plan_EXHAUSTIVE_SOURCE_PASS.xlsx
+++ b/docs/FoxESS_PQ1_Register_Mapping_and_Test_Plan_EXHAUSTIVE_SOURCE_PASS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paul/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paul/dev/foxess_modbus/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_FDC73781CF48E09F47B24D0280233368A978CD6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4627E6B8-B18D-AD48-B2FE-933949E8961A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Mapping" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1837" uniqueCount="850">
   <si>
     <t>Register/Register Range</t>
   </si>
@@ -2253,6 +2253,373 @@
   </si>
   <si>
     <t>Read-only; no remote writes.</t>
+  </si>
+  <si>
+    <t>PR1 implementation plan (not yet implemented)</t>
+  </si>
+  <si>
+    <t>Proposed Home Assistant sensor names (read-only)</t>
+  </si>
+  <si>
+    <t>Proposed HA domain.key (configured prefix omitted)</t>
+  </si>
+  <si>
+    <t>No — deferred / unresolved</t>
+  </si>
+  <si>
+    <t>None in PR1</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Yes — planned, read-only</t>
+  </si>
+  <si>
+    <t>Grid Voltage</t>
+  </si>
+  <si>
+    <t>sensor.rvolt</t>
+  </si>
+  <si>
+    <t>Inverter Current</t>
+  </si>
+  <si>
+    <t>sensor.rcurrent</t>
+  </si>
+  <si>
+    <t>Inverter Power</t>
+  </si>
+  <si>
+    <t>sensor.rpower</t>
+  </si>
+  <si>
+    <t>EPS Voltage</t>
+  </si>
+  <si>
+    <t>sensor.eps_rvolt</t>
+  </si>
+  <si>
+    <t>Conditional — verify scaling and flow direction</t>
+  </si>
+  <si>
+    <t>Grid CT
+Feed-in
+Grid Consumption</t>
+  </si>
+  <si>
+    <t>sensor.grid_ct
+sensor.feed_in
+sensor.grid_consumption</t>
+  </si>
+  <si>
+    <t>Load Power</t>
+  </si>
+  <si>
+    <t>sensor.load_power</t>
+  </si>
+  <si>
+    <t>Partial — only 31022 and 31024; see individual rows</t>
+  </si>
+  <si>
+    <t>Inverter Battery Power; Battery Charge / Discharge; Battery SoC</t>
+  </si>
+  <si>
+    <t>sensor.invbatpower
+sensor.battery_charge
+sensor.battery_discharge
+sensor.battery_soc</t>
+  </si>
+  <si>
+    <t>Inverter Battery Power
+Battery Charge
+Battery Discharge</t>
+  </si>
+  <si>
+    <t>sensor.invbatpower
+sensor.battery_charge
+sensor.battery_discharge</t>
+  </si>
+  <si>
+    <t>Battery SoC</t>
+  </si>
+  <si>
+    <t>sensor.battery_soc</t>
+  </si>
+  <si>
+    <t>Conditional — validate individual counters and scales; candidate register assignments shown</t>
+  </si>
+  <si>
+    <t>32000–01: Solar Generation Total
+32002: Solar Generation Today
+32003–04: Battery Charge Total
+32005: Battery Charge Today
+32006–07: Battery Discharge Total
+32008: Battery Discharge Today
+32009–10: Feed-in Total
+32011: Feed-in Today
+32012–13: Grid Consumption Total
+32014: Grid Consumption Today
+32015–16: Yield Total
+32017: Yield Today
+32018–19: Input Energy Total
+32020: Input Energy Today
+32021–22: Load Energy Total
+32023: Load Energy Today</t>
+  </si>
+  <si>
+    <t>sensor.solar_energy_total
+sensor.solar_energy_today
+sensor.battery_charge_total
+sensor.battery_charge_today
+sensor.battery_discharge_total
+sensor.battery_discharge_today
+sensor.feed_in_energy_total
+sensor.feed_in_energy_today
+sensor.grid_consumption_energy_total
+sensor.grid_consumption_energy_today
+sensor.total_yield_total
+sensor.total_yield_today
+sensor.input_energy_total
+sensor.input_energy_today
+sensor.load_power_total
+sensor.load_energy_today</t>
+  </si>
+  <si>
+    <t>Version: Master</t>
+  </si>
+  <si>
+    <t>sensor.master_version</t>
+  </si>
+  <si>
+    <t>Version: Slave</t>
+  </si>
+  <si>
+    <t>sensor.slave_version</t>
+  </si>
+  <si>
+    <t>Version: Manager</t>
+  </si>
+  <si>
+    <t>sensor.manager_version</t>
+  </si>
+  <si>
+    <t>Conditional — verify BMS meanings and scales</t>
+  </si>
+  <si>
+    <t>37609: Battery Voltage
+37610: Battery Current</t>
+  </si>
+  <si>
+    <t>sensor.batvolt
+sensor.bat_current</t>
+  </si>
+  <si>
+    <t>Conditional — verify temperature meaning and scale</t>
+  </si>
+  <si>
+    <t>Battery Temp</t>
+  </si>
+  <si>
+    <t>sensor.battery_temp</t>
+  </si>
+  <si>
+    <t>37617: BMS Cell Temp High
+37618: BMS Cell Temp Low
+37619: BMS Cell mV High
+37620: BMS Cell mV Low</t>
+  </si>
+  <si>
+    <t>sensor.bms_cell_temp_high
+sensor.bms_cell_temp_low
+sensor.bms_cell_mv_high
+sensor.bms_cell_mv_low</t>
+  </si>
+  <si>
+    <t>Battery SoH</t>
+  </si>
+  <si>
+    <t>sensor.battery_soh</t>
+  </si>
+  <si>
+    <t>BMS kWh Remaining</t>
+  </si>
+  <si>
+    <t>sensor.bms_kwh_remaining</t>
+  </si>
+  <si>
+    <t>No — status/fault decoding needs PQ1 evidence</t>
+  </si>
+  <si>
+    <t>PV1 Voltage</t>
+  </si>
+  <si>
+    <t>sensor.pv1_voltage</t>
+  </si>
+  <si>
+    <t>PV1 Current</t>
+  </si>
+  <si>
+    <t>sensor.pv1_current</t>
+  </si>
+  <si>
+    <t>PV2 Voltage</t>
+  </si>
+  <si>
+    <t>sensor.pv2_voltage</t>
+  </si>
+  <si>
+    <t>PV2 Current</t>
+  </si>
+  <si>
+    <t>sensor.pv2_current</t>
+  </si>
+  <si>
+    <t>PV3 Voltage</t>
+  </si>
+  <si>
+    <t>sensor.pv3_voltage</t>
+  </si>
+  <si>
+    <t>PV3 Current</t>
+  </si>
+  <si>
+    <t>sensor.pv3_current</t>
+  </si>
+  <si>
+    <t>PV4 Voltage</t>
+  </si>
+  <si>
+    <t>sensor.pv4_voltage</t>
+  </si>
+  <si>
+    <t>PV4 Current</t>
+  </si>
+  <si>
+    <t>sensor.pv4_current</t>
+  </si>
+  <si>
+    <t>PV Power</t>
+  </si>
+  <si>
+    <t>sensor.pv_power_now</t>
+  </si>
+  <si>
+    <t>No — use 31006 for PR1</t>
+  </si>
+  <si>
+    <t>None from this register; Grid Voltage uses 31006</t>
+  </si>
+  <si>
+    <t>No — use 31007 for PR1</t>
+  </si>
+  <si>
+    <t>None from this register; Inverter Current uses 31007</t>
+  </si>
+  <si>
+    <t>No — unresolved alternative; use 31008 in PR1</t>
+  </si>
+  <si>
+    <t>None from this register/pair; Inverter Power uses 31008</t>
+  </si>
+  <si>
+    <t>Grid Frequency</t>
+  </si>
+  <si>
+    <t>sensor.rfreq</t>
+  </si>
+  <si>
+    <t>Inverter Temp</t>
+  </si>
+  <si>
+    <t>sensor.invtemp</t>
+  </si>
+  <si>
+    <t>Conditional — confirm 16/32-bit width and word order</t>
+  </si>
+  <si>
+    <t>PV1 Power</t>
+  </si>
+  <si>
+    <t>sensor.pv1_power</t>
+  </si>
+  <si>
+    <t>PV2 Power</t>
+  </si>
+  <si>
+    <t>sensor.pv2_power</t>
+  </si>
+  <si>
+    <t>PV3 Power</t>
+  </si>
+  <si>
+    <t>sensor.pv3_power</t>
+  </si>
+  <si>
+    <t>PV4 Power</t>
+  </si>
+  <si>
+    <t>sensor.pv4_power</t>
+  </si>
+  <si>
+    <t>Yes — planned read-only; label only confirmed mode values</t>
+  </si>
+  <si>
+    <t>Manual Work Mode</t>
+  </si>
+  <si>
+    <t>sensor.manual_work_mode (proposed new key)</t>
+  </si>
+  <si>
+    <t>Max Charge Current</t>
+  </si>
+  <si>
+    <t>sensor.max_charge_current</t>
+  </si>
+  <si>
+    <t>Max Discharge Current</t>
+  </si>
+  <si>
+    <t>sensor.max_discharge_current</t>
+  </si>
+  <si>
+    <t>Min SoC</t>
+  </si>
+  <si>
+    <t>sensor.min_soc</t>
+  </si>
+  <si>
+    <t>Max SoC</t>
+  </si>
+  <si>
+    <t>sensor.max_soc</t>
+  </si>
+  <si>
+    <t>Min SoC (On Grid)</t>
+  </si>
+  <si>
+    <t>sensor.min_soc_on_grid</t>
+  </si>
+  <si>
+    <t>No — use corresponding 41007–41011 register</t>
+  </si>
+  <si>
+    <t>None from duplicate map in PR1</t>
+  </si>
+  <si>
+    <t>No — deferred pending controlled export-limit validation</t>
+  </si>
+  <si>
+    <t>None in current PR1 scope</t>
+  </si>
+  <si>
+    <t>Scheduler Enabled</t>
+  </si>
+  <si>
+    <t>binary_sensor.scheduler_enabled (proposed new key)</t>
+  </si>
+  <si>
+    <t>No — scheduler parsing deferred to PR3</t>
   </si>
 </sst>
 </file>
@@ -2384,9 +2751,9 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="PQ1 status of meaning"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Format/scaling"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="R RW (R,RW)"/>
-    <tableColumn id="9" name="PR1 implementation plan (not yet implemented)"/>
-    <tableColumn id="10" name="Proposed Home Assistant sensor names (read-only)"/>
-    <tableColumn id="11" name="Proposed HA domain.key (configured prefix omitted)"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="PR1 implementation plan (not yet implemented)"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proposed Home Assistant sensor names (read-only)"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Proposed HA domain.key (configured prefix omitted)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2643,20 +3010,14 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PR1 implementation plan (not yet implemented)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposed Home Assistant sensor names (read-only)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposed HA domain.key (configured prefix omitted)</t>
-        </is>
+      <c r="I1" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>746</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="45.25" customHeight="1">
@@ -2684,20 +3045,14 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I2" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="45.25" customHeight="1">
@@ -2725,20 +3080,14 @@
       <c r="H3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I3" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="45.25" customHeight="1">
@@ -2766,20 +3115,14 @@
       <c r="H4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grid Voltage</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.rvolt</t>
-        </is>
+      <c r="I4" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>751</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>752</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="45.25" customHeight="1">
@@ -2807,20 +3150,14 @@
       <c r="H5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inverter Current</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.rcurrent</t>
-        </is>
+      <c r="I5" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>753</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>754</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="45.25" customHeight="1">
@@ -2848,20 +3185,14 @@
       <c r="H6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inverter Power</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.rpower</t>
-        </is>
+      <c r="I6" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>755</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>756</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="45.25" customHeight="1">
@@ -2889,20 +3220,14 @@
       <c r="H7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EPS Voltage</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.eps_rvolt</t>
-        </is>
+      <c r="I7" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>757</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>758</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="48" customHeight="1">
@@ -2930,24 +3255,14 @@
       <c r="H8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conditional — verify scaling and flow direction</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grid CT
-Feed-in
-Grid Consumption</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.grid_ct
-sensor.feed_in
-sensor.grid_consumption</t>
-        </is>
+      <c r="I8" s="3" t="s">
+        <v>759</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>761</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="45.25" customHeight="1">
@@ -2975,20 +3290,14 @@
       <c r="H9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I9" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="45.25" customHeight="1">
@@ -3016,20 +3325,14 @@
       <c r="H10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Load Power</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.load_power</t>
-        </is>
+      <c r="I10" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>762</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>763</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="45.25" customHeight="1">
@@ -3057,20 +3360,14 @@
       <c r="H11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I11" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="62" customHeight="1">
@@ -3098,23 +3395,14 @@
       <c r="H12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial — only 31022 and 31024; see individual rows</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inverter Battery Power; Battery Charge / Discharge; Battery SoC</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.invbatpower
-sensor.battery_charge
-sensor.battery_discharge
-sensor.battery_soc</t>
-        </is>
+      <c r="I12" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>766</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="48" customHeight="1">
@@ -3142,24 +3430,14 @@
       <c r="H13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inverter Battery Power
-Battery Charge
-Battery Discharge</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.invbatpower
-sensor.battery_charge
-sensor.battery_discharge</t>
-        </is>
+      <c r="I13" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>767</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>768</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="45.25" customHeight="1">
@@ -3187,20 +3465,14 @@
       <c r="H14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Battery SoC</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.battery_soc</t>
-        </is>
+      <c r="I14" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>770</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="45.25" customHeight="1">
@@ -3228,20 +3500,14 @@
       <c r="H15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I15" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="45.25" customHeight="1">
@@ -3269,20 +3535,14 @@
       <c r="H16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I16" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="45.25" customHeight="1">
@@ -3310,20 +3570,14 @@
       <c r="H17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I17" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="230" customHeight="1">
@@ -3351,50 +3605,14 @@
       <c r="H18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conditional — validate individual counters and scales; candidate register assignments shown</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32000–01: Solar Generation Total
-32002: Solar Generation Today
-32003–04: Battery Charge Total
-32005: Battery Charge Today
-32006–07: Battery Discharge Total
-32008: Battery Discharge Today
-32009–10: Feed-in Total
-32011: Feed-in Today
-32012–13: Grid Consumption Total
-32014: Grid Consumption Today
-32015–16: Yield Total
-32017: Yield Today
-32018–19: Input Energy Total
-32020: Input Energy Today
-32021–22: Load Energy Total
-32023: Load Energy Today</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.solar_energy_total
-sensor.solar_energy_today
-sensor.battery_charge_total
-sensor.battery_charge_today
-sensor.battery_discharge_total
-sensor.battery_discharge_today
-sensor.feed_in_energy_total
-sensor.feed_in_energy_today
-sensor.grid_consumption_energy_total
-sensor.grid_consumption_energy_today
-sensor.total_yield_total
-sensor.total_yield_today
-sensor.input_energy_total
-sensor.input_energy_today
-sensor.load_power_total
-sensor.load_energy_today</t>
-        </is>
+      <c r="I18" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>772</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>773</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="45.25" customHeight="1">
@@ -3422,20 +3640,14 @@
       <c r="H19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Version: Master</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.master_version</t>
-        </is>
+      <c r="I19" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>775</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="45.25" customHeight="1">
@@ -3463,20 +3675,14 @@
       <c r="H20" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Version: Slave</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.slave_version</t>
-        </is>
+      <c r="I20" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>776</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>777</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="45.25" customHeight="1">
@@ -3504,20 +3710,14 @@
       <c r="H21" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Version: Manager</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.manager_version</t>
-        </is>
+      <c r="I21" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>779</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="45.25" customHeight="1">
@@ -3545,20 +3745,14 @@
       <c r="H22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I22" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="45.25" customHeight="1">
@@ -3586,22 +3780,14 @@
       <c r="H23" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conditional — verify BMS meanings and scales</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">37609: Battery Voltage
-37610: Battery Current</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.batvolt
-sensor.bat_current</t>
-        </is>
+      <c r="I23" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>782</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="45.25" customHeight="1">
@@ -3629,20 +3815,14 @@
       <c r="H24" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conditional — verify temperature meaning and scale</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Battery Temp</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.battery_temp</t>
-        </is>
+      <c r="I24" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>785</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="62" customHeight="1">
@@ -3670,26 +3850,14 @@
       <c r="H25" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">37617: BMS Cell Temp High
-37618: BMS Cell Temp Low
-37619: BMS Cell mV High
-37620: BMS Cell mV Low</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.bms_cell_temp_high
-sensor.bms_cell_temp_low
-sensor.bms_cell_mv_high
-sensor.bms_cell_mv_low</t>
-        </is>
+      <c r="I25" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>787</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="45.25" customHeight="1">
@@ -3717,20 +3885,14 @@
       <c r="H26" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Battery SoH</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.battery_soh</t>
-        </is>
+      <c r="I26" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>789</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="45.25" customHeight="1">
@@ -3758,20 +3920,14 @@
       <c r="H27" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BMS kWh Remaining</t>
-        </is>
-      </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.bms_kwh_remaining</t>
-        </is>
+      <c r="I27" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>791</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="45.25" customHeight="1">
@@ -3799,20 +3955,14 @@
       <c r="H28" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — status/fault decoding needs PQ1 evidence</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I28" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="45.25" customHeight="1">
@@ -3840,20 +3990,14 @@
       <c r="H29" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — status/fault decoding needs PQ1 evidence</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I29" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="45.25" customHeight="1">
@@ -3881,20 +4025,14 @@
       <c r="H30" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV1 Voltage</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv1_voltage</t>
-        </is>
+      <c r="I30" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>793</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="45.25" customHeight="1">
@@ -3922,20 +4060,14 @@
       <c r="H31" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV1 Current</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv1_current</t>
-        </is>
+      <c r="I31" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>796</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="45.25" customHeight="1">
@@ -3963,20 +4095,14 @@
       <c r="H32" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV2 Voltage</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv2_voltage</t>
-        </is>
+      <c r="I32" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>798</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="45.25" customHeight="1">
@@ -4004,20 +4130,14 @@
       <c r="H33" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV2 Current</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv2_current</t>
-        </is>
+      <c r="I33" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>800</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="45.25" customHeight="1">
@@ -4045,20 +4165,14 @@
       <c r="H34" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV3 Voltage</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv3_voltage</t>
-        </is>
+      <c r="I34" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>801</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>802</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="45.25" customHeight="1">
@@ -4086,20 +4200,14 @@
       <c r="H35" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV3 Current</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv3_current</t>
-        </is>
+      <c r="I35" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>804</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="45.25" customHeight="1">
@@ -4127,20 +4235,14 @@
       <c r="H36" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV4 Voltage</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv4_voltage</t>
-        </is>
+      <c r="I36" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>806</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="45.25" customHeight="1">
@@ -4168,20 +4270,14 @@
       <c r="H37" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV4 Current</t>
-        </is>
-      </c>
-      <c r="K37" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv4_current</t>
-        </is>
+      <c r="I37" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>808</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="45.25" customHeight="1">
@@ -4209,20 +4305,14 @@
       <c r="H38" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV Power</t>
-        </is>
-      </c>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv_power_now</t>
-        </is>
+      <c r="I38" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>810</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="45.25" customHeight="1">
@@ -4250,20 +4340,14 @@
       <c r="H39" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — use 31006 for PR1</t>
-        </is>
-      </c>
-      <c r="J39" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from this register; Grid Voltage uses 31006</t>
-        </is>
-      </c>
-      <c r="K39" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I39" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>812</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="45.25" customHeight="1">
@@ -4291,20 +4375,14 @@
       <c r="H40" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I40" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — use 31007 for PR1</t>
-        </is>
-      </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from this register; Inverter Current uses 31007</t>
-        </is>
-      </c>
-      <c r="K40" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I40" s="3" t="s">
+        <v>813</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="45.25" customHeight="1">
@@ -4332,20 +4410,14 @@
       <c r="H41" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — unresolved alternative; use 31008 in PR1</t>
-        </is>
-      </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from this register/pair; Inverter Power uses 31008</t>
-        </is>
-      </c>
-      <c r="K41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I41" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>816</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="45.25" customHeight="1">
@@ -4373,20 +4445,14 @@
       <c r="H42" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grid Frequency</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.rfreq</t>
-        </is>
+      <c r="I42" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>817</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>818</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="45.25" customHeight="1">
@@ -4414,20 +4480,14 @@
       <c r="H43" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inverter Temp</t>
-        </is>
-      </c>
-      <c r="K43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.invtemp</t>
-        </is>
+      <c r="I43" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>820</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="45.25" customHeight="1">
@@ -4455,20 +4515,14 @@
       <c r="H44" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I44" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K44" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I44" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="45.25" customHeight="1">
@@ -4496,20 +4550,14 @@
       <c r="H45" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I45" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J45" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K45" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I45" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K45" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="45.25" customHeight="1">
@@ -4537,20 +4585,14 @@
       <c r="H46" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I46" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J46" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K46" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I46" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="45.25" customHeight="1">
@@ -4578,20 +4620,14 @@
       <c r="H47" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I47" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J47" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K47" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I47" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J47" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K47" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="45.25" customHeight="1">
@@ -4619,20 +4655,14 @@
       <c r="H48" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I48" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J48" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K48" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I48" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K48" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="45.25" customHeight="1">
@@ -4660,20 +4690,14 @@
       <c r="H49" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I49" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J49" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K49" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I49" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K49" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="45.25" customHeight="1">
@@ -4701,20 +4725,14 @@
       <c r="H50" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J50" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K50" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I50" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="45.25" customHeight="1">
@@ -4742,20 +4760,14 @@
       <c r="H51" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I51" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K51" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="45.25" customHeight="1">
@@ -4783,20 +4795,14 @@
       <c r="H52" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I52" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conditional — confirm 16/32-bit width and word order</t>
-        </is>
-      </c>
-      <c r="J52" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV1 Power</t>
-        </is>
-      </c>
-      <c r="K52" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv1_power</t>
-        </is>
+      <c r="I52" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>822</v>
+      </c>
+      <c r="K52" s="3" t="s">
+        <v>823</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="45.25" customHeight="1">
@@ -4824,20 +4830,14 @@
       <c r="H53" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conditional — confirm 16/32-bit width and word order</t>
-        </is>
-      </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV2 Power</t>
-        </is>
-      </c>
-      <c r="K53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv2_power</t>
-        </is>
+      <c r="I53" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>824</v>
+      </c>
+      <c r="K53" s="3" t="s">
+        <v>825</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="45.25" customHeight="1">
@@ -4865,20 +4865,14 @@
       <c r="H54" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I54" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conditional — confirm 16/32-bit width and word order</t>
-        </is>
-      </c>
-      <c r="J54" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV3 Power</t>
-        </is>
-      </c>
-      <c r="K54" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv3_power</t>
-        </is>
+      <c r="I54" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="J54" s="3" t="s">
+        <v>826</v>
+      </c>
+      <c r="K54" s="3" t="s">
+        <v>827</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="45.25" customHeight="1">
@@ -4906,20 +4900,14 @@
       <c r="H55" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conditional — confirm 16/32-bit width and word order</t>
-        </is>
-      </c>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV4 Power</t>
-        </is>
-      </c>
-      <c r="K55" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.pv4_power</t>
-        </is>
+      <c r="I55" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="J55" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="K55" s="3" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="45.25" customHeight="1">
@@ -4947,20 +4935,14 @@
       <c r="H56" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I56" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned read-only; label only confirmed mode values</t>
-        </is>
-      </c>
-      <c r="J56" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manual Work Mode</t>
-        </is>
-      </c>
-      <c r="K56" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.manual_work_mode (proposed new key)</t>
-        </is>
+      <c r="I56" s="3" t="s">
+        <v>830</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="K56" s="3" t="s">
+        <v>832</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="45.25" customHeight="1">
@@ -4988,20 +4970,14 @@
       <c r="H57" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I57" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J57" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Max Charge Current</t>
-        </is>
-      </c>
-      <c r="K57" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.max_charge_current</t>
-        </is>
+      <c r="I57" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J57" s="3" t="s">
+        <v>833</v>
+      </c>
+      <c r="K57" s="3" t="s">
+        <v>834</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="45.25" customHeight="1">
@@ -5029,20 +5005,14 @@
       <c r="H58" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Max Discharge Current</t>
-        </is>
-      </c>
-      <c r="K58" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.max_discharge_current</t>
-        </is>
+      <c r="I58" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J58" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="K58" s="3" t="s">
+        <v>836</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="45.25" customHeight="1">
@@ -5070,20 +5040,14 @@
       <c r="H59" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Min SoC</t>
-        </is>
-      </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.min_soc</t>
-        </is>
+      <c r="I59" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J59" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="K59" s="3" t="s">
+        <v>838</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="45.25" customHeight="1">
@@ -5111,20 +5075,14 @@
       <c r="H60" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J60" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Max SoC</t>
-        </is>
-      </c>
-      <c r="K60" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.max_soc</t>
-        </is>
+      <c r="I60" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J60" s="3" t="s">
+        <v>839</v>
+      </c>
+      <c r="K60" s="3" t="s">
+        <v>840</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="45.25" customHeight="1">
@@ -5152,20 +5110,14 @@
       <c r="H61" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Min SoC (On Grid)</t>
-        </is>
-      </c>
-      <c r="K61" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor.min_soc_on_grid</t>
-        </is>
+      <c r="I61" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J61" s="3" t="s">
+        <v>841</v>
+      </c>
+      <c r="K61" s="3" t="s">
+        <v>842</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="45.25" customHeight="1">
@@ -5193,20 +5145,14 @@
       <c r="H62" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I62" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J62" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K62" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I62" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J62" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K62" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="45.25" customHeight="1">
@@ -5234,20 +5180,14 @@
       <c r="H63" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I63" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K63" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I63" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J63" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K63" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="45.25" customHeight="1">
@@ -5275,20 +5215,14 @@
       <c r="H64" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K64" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I64" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J64" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K64" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="45.25" customHeight="1">
@@ -5316,20 +5250,14 @@
       <c r="H65" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="I65" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J65" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K65" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I65" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J65" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K65" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="66" spans="1:11" ht="45.25" customHeight="1">
@@ -5357,20 +5285,14 @@
       <c r="H66" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — use corresponding 41007–41011 register</t>
-        </is>
-      </c>
-      <c r="J66" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from duplicate map in PR1</t>
-        </is>
-      </c>
-      <c r="K66" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I66" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="J66" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="K66" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="45.25" customHeight="1">
@@ -5398,20 +5320,14 @@
       <c r="H67" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — use corresponding 41007–41011 register</t>
-        </is>
-      </c>
-      <c r="J67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from duplicate map in PR1</t>
-        </is>
-      </c>
-      <c r="K67" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I67" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="J67" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="K67" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="68" spans="1:11" ht="45.25" customHeight="1">
@@ -5439,20 +5355,14 @@
       <c r="H68" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I68" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — use corresponding 41007–41011 register</t>
-        </is>
-      </c>
-      <c r="J68" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from duplicate map in PR1</t>
-        </is>
-      </c>
-      <c r="K68" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I68" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="J68" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="K68" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="45.25" customHeight="1">
@@ -5480,20 +5390,14 @@
       <c r="H69" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — use corresponding 41007–41011 register</t>
-        </is>
-      </c>
-      <c r="J69" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from duplicate map in PR1</t>
-        </is>
-      </c>
-      <c r="K69" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I69" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="J69" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="K69" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="70" spans="1:11" ht="45.25" customHeight="1">
@@ -5521,20 +5425,14 @@
       <c r="H70" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I70" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — use corresponding 41007–41011 register</t>
-        </is>
-      </c>
-      <c r="J70" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from duplicate map in PR1</t>
-        </is>
-      </c>
-      <c r="K70" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I70" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="J70" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="K70" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="71" spans="1:11" ht="45.25" customHeight="1">
@@ -5562,20 +5460,14 @@
       <c r="H71" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I71" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred pending controlled export-limit validation</t>
-        </is>
-      </c>
-      <c r="J71" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in current PR1 scope</t>
-        </is>
-      </c>
-      <c r="K71" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I71" s="3" t="s">
+        <v>845</v>
+      </c>
+      <c r="J71" s="3" t="s">
+        <v>846</v>
+      </c>
+      <c r="K71" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="72" spans="1:11" ht="45.25" customHeight="1">
@@ -5603,20 +5495,14 @@
       <c r="H72" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I72" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J72" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K72" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I72" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J72" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K72" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="45.25" customHeight="1">
@@ -5644,20 +5530,14 @@
       <c r="H73" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I73" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes — planned, read-only</t>
-        </is>
-      </c>
-      <c r="J73" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Scheduler Enabled</t>
-        </is>
-      </c>
-      <c r="K73" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">binary_sensor.scheduler_enabled (proposed new key)</t>
-        </is>
+      <c r="I73" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="J73" s="3" t="s">
+        <v>847</v>
+      </c>
+      <c r="K73" s="3" t="s">
+        <v>848</v>
       </c>
     </row>
     <row r="74" spans="1:11" ht="45.25" customHeight="1">
@@ -5685,20 +5565,14 @@
       <c r="H74" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I74" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J74" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K74" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I74" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K74" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="75" spans="1:11" ht="45.25" customHeight="1">
@@ -5726,20 +5600,14 @@
       <c r="H75" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I75" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J75" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K75" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I75" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K75" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="76" spans="1:11" ht="45.25" customHeight="1">
@@ -5767,20 +5635,14 @@
       <c r="H76" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I76" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J76" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K76" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I76" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J76" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K76" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="77" spans="1:11" ht="45.25" customHeight="1">
@@ -5808,20 +5670,14 @@
       <c r="H77" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I77" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J77" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K77" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I77" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J77" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K77" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="78" spans="1:11" ht="45.25" customHeight="1">
@@ -5849,20 +5705,14 @@
       <c r="H78" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I78" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J78" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K78" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I78" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J78" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K78" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="79" spans="1:11" ht="45.25" customHeight="1">
@@ -5890,20 +5740,14 @@
       <c r="H79" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I79" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J79" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K79" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I79" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K79" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="45.25" customHeight="1">
@@ -5931,20 +5775,14 @@
       <c r="H80" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I80" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J80" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K80" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I80" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J80" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K80" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="45.25" customHeight="1">
@@ -5972,20 +5810,14 @@
       <c r="H81" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I81" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J81" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K81" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I81" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J81" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K81" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="82" spans="1:11" ht="45.25" customHeight="1">
@@ -6013,20 +5845,14 @@
       <c r="H82" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I82" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J82" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K82" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I82" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J82" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K82" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="45.25" customHeight="1">
@@ -6054,20 +5880,14 @@
       <c r="H83" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I83" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J83" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K83" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I83" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J83" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K83" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="45.25" customHeight="1">
@@ -6095,20 +5915,14 @@
       <c r="H84" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I84" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — scheduler parsing deferred to PR3</t>
-        </is>
-      </c>
-      <c r="J84" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K84" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I84" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="J84" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K84" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="45.25" customHeight="1">
@@ -6136,20 +5950,14 @@
       <c r="H85" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I85" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J85" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K85" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="45.25" customHeight="1">
@@ -6177,20 +5985,14 @@
       <c r="H86" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I86" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J86" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K86" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I86" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J86" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K86" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="45.25" customHeight="1">
@@ -6218,20 +6020,14 @@
       <c r="H87" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I87" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J87" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K87" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I87" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J87" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K87" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="45.25" customHeight="1">
@@ -6259,20 +6055,14 @@
       <c r="H88" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I88" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J88" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K88" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I88" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J88" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K88" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="45.25" customHeight="1">
@@ -6300,20 +6090,14 @@
       <c r="H89" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I89" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J89" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K89" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I89" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="J89" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="K89" s="3" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="45">
@@ -6341,20 +6125,14 @@
       <c r="H90" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I90" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J90" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K90" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I90" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J90" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K90" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="45">
@@ -6382,20 +6160,14 @@
       <c r="H91" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I91" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J91" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K91" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I91" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J91" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K91" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="45">
@@ -6423,20 +6195,14 @@
       <c r="H92" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I92" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — unresolved alternative; use 31008 in PR1</t>
-        </is>
-      </c>
-      <c r="J92" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None from this register/pair; Inverter Power uses 31008</t>
-        </is>
-      </c>
-      <c r="K92" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I92" s="2" t="s">
+        <v>815</v>
+      </c>
+      <c r="J92" s="2" t="s">
+        <v>816</v>
+      </c>
+      <c r="K92" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="30">
@@ -6464,20 +6230,14 @@
       <c r="H93" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I93" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J93" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K93" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I93" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J93" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K93" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="30">
@@ -6505,20 +6265,14 @@
       <c r="H94" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I94" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J94" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K94" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I94" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K94" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="30">
@@ -6546,20 +6300,14 @@
       <c r="H95" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I95" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J95" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K95" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I95" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J95" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K95" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="30">
@@ -6587,20 +6335,14 @@
       <c r="H96" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I96" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J96" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K96" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I96" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J96" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K96" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="30">
@@ -6628,20 +6370,14 @@
       <c r="H97" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I97" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J97" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K97" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I97" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J97" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K97" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="30">
@@ -6669,20 +6405,14 @@
       <c r="H98" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I98" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J98" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K98" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I98" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K98" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="30">
@@ -6710,20 +6440,14 @@
       <c r="H99" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I99" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J99" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K99" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I99" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J99" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K99" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="45">
@@ -6751,20 +6475,14 @@
       <c r="H100" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I100" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J100" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K100" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I100" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K100" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="45">
@@ -6792,20 +6510,14 @@
       <c r="H101" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I101" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J101" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K101" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I101" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J101" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K101" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="102" spans="1:11" ht="30">
@@ -6833,20 +6545,14 @@
       <c r="H102" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I102" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J102" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K102" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I102" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J102" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K102" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="45">
@@ -6874,20 +6580,14 @@
       <c r="H103" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I103" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J103" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K103" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I103" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J103" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K103" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="45">
@@ -6915,20 +6615,14 @@
       <c r="H104" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I104" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J104" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K104" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I104" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J104" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K104" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="60">
@@ -6956,20 +6650,14 @@
       <c r="H105" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I105" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J105" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K105" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I105" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J105" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K105" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="106" spans="1:11" ht="30">
@@ -6997,20 +6685,14 @@
       <c r="H106" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I106" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J106" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K106" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I106" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J106" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K106" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="30">
@@ -7038,20 +6720,14 @@
       <c r="H107" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I107" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J107" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K107" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I107" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J107" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K107" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="30">
@@ -7079,20 +6755,14 @@
       <c r="H108" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I108" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J108" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K108" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I108" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J108" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K108" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="30">
@@ -7120,20 +6790,14 @@
       <c r="H109" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I109" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J109" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K109" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I109" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J109" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K109" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="30">
@@ -7161,20 +6825,14 @@
       <c r="H110" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I110" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J110" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K110" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I110" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J110" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K110" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="30">
@@ -7202,20 +6860,14 @@
       <c r="H111" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I111" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J111" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K111" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I111" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J111" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K111" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="30">
@@ -7243,20 +6895,14 @@
       <c r="H112" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I112" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J112" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K112" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I112" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J112" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K112" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="30">
@@ -7284,23 +6930,17 @@
       <c r="H113" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I113" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J113" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K113" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" spans="1:11" ht="20">
+      <c r="I113" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J113" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K113" s="2" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" ht="15">
       <c r="A114" s="2" t="s">
         <v>452</v>
       </c>
@@ -7325,20 +6965,14 @@
       <c r="H114" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I114" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J114" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K114" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I114" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J114" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K114" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="115" spans="1:11" ht="30">
@@ -7366,20 +7000,14 @@
       <c r="H115" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I115" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J115" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K115" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I115" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J115" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K115" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="116" spans="1:11" ht="45">
@@ -7407,20 +7035,14 @@
       <c r="H116" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I116" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J116" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K116" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I116" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J116" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K116" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="117" spans="1:11" ht="45">
@@ -7448,20 +7070,14 @@
       <c r="H117" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I117" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J117" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K117" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I117" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J117" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K117" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="118" spans="1:11" ht="30">
@@ -7489,20 +7105,14 @@
       <c r="H118" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I118" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J118" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K118" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I118" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J118" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K118" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="119" spans="1:11" ht="45">
@@ -7530,20 +7140,14 @@
       <c r="H119" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I119" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J119" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K119" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I119" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J119" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K119" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="120" spans="1:11" ht="30">
@@ -7571,20 +7175,14 @@
       <c r="H120" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I120" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J120" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K120" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I120" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J120" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K120" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="121" spans="1:11" ht="30">
@@ -7612,20 +7210,14 @@
       <c r="H121" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I121" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J121" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K121" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I121" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J121" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K121" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="122" spans="1:11" ht="30">
@@ -7653,20 +7245,14 @@
       <c r="H122" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I122" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J122" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K122" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="123" spans="1:11" ht="30">
@@ -7694,20 +7280,14 @@
       <c r="H123" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I123" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J123" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K123" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="124" spans="1:11" ht="30">
@@ -7735,20 +7315,14 @@
       <c r="H124" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I124" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J124" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K124" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="125" spans="1:11" ht="30">
@@ -7776,20 +7350,14 @@
       <c r="H125" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I125" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J125" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K125" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="126" spans="1:11" ht="45">
@@ -7817,20 +7385,14 @@
       <c r="H126" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I126" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J126" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K126" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="45">
@@ -7858,20 +7420,14 @@
       <c r="H127" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I127" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J127" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K127" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="30">
@@ -7899,20 +7455,14 @@
       <c r="H128" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I128" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J128" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K128" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="30">
@@ -7940,20 +7490,14 @@
       <c r="H129" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I129" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J129" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K129" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="130" spans="1:11" ht="30">
@@ -7981,20 +7525,14 @@
       <c r="H130" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I130" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J130" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K130" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="131" spans="1:11" ht="30">
@@ -8022,20 +7560,14 @@
       <c r="H131" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I131" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J131" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K131" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="132" spans="1:11" ht="30">
@@ -8063,20 +7595,14 @@
       <c r="H132" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I132" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J132" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K132" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="133" spans="1:11" ht="30">
@@ -8104,20 +7630,14 @@
       <c r="H133" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I133" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J133" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K133" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="134" spans="1:11" ht="30">
@@ -8145,20 +7665,14 @@
       <c r="H134" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I134" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J134" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K134" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="135" spans="1:11" ht="45">
@@ -8186,20 +7700,14 @@
       <c r="H135" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No — deferred / unresolved</t>
-        </is>
-      </c>
-      <c r="J135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None in PR1</t>
-        </is>
-      </c>
-      <c r="K135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="I135" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="J135" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="K135" s="2" t="s">
+        <v>749</v>
       </c>
     </row>
   </sheetData>

</xml_diff>